<commit_message>
Fix RA_Kasalis: only real operator-accessible tasks under normal operation
Removed the torna-mesa / gantry dispensador / gantry PnP rows from
"operacion normal" -- the operator has no physical access to those
mechanisms during the automatic cycle (they sit behind the safety
curtains/guards), so that hazard only applies to maintenance with
interlocks bypassed. Consolidated it into one maintenance row instead.

Normal operation now lists what the operator actually does: carga de
material, descarga de material, limpieza de la maquina, manejo de
materiales (ergonomia), and chemical residue contact -- 8 rows total
(was 9). Standardized the "documento" field to 16-AT40-3318-00005
across all rows per user request.
</commit_message>
<xml_diff>
--- a/moc_2406/RA_Kasalis.xlsx
+++ b/moc_2406/RA_Kasalis.xlsx
@@ -6606,12 +6606,12 @@
       </c>
       <c r="B8" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operación normal - rotación de la torna-mesa (4 estaciones)</t>
+          <t xml:space="preserve">Operación normal - carga de material en la estación con contacto directo del operador</t>
         </is>
       </c>
       <c r="C8" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">La torna-mesa gira mediante un motor de gran tamaño para posicionar cada estación frente a los gantries de dispensado/PnP</t>
+          <t xml:space="preserve">El operador coloca la pieza en la estación de carga; al hacerlo se activa el pistón de clampeo que asegura la pieza. Es el punto de mayor riesgo de la máquina por el contacto directo del operador con el mecanismo.</t>
         </is>
       </c>
       <c r="D8" s="56" t="inlineStr">
@@ -6626,7 +6626,7 @@
       </c>
       <c r="F8" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Atrapamiento</t>
+          <t xml:space="preserve">Amputación</t>
         </is>
       </c>
       <c r="G8" s="56" t="inlineStr">
@@ -6636,7 +6636,7 @@
       </c>
       <c r="H8" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="I8" s="57" t="inlineStr">
@@ -6655,12 +6655,12 @@
       </c>
       <c r="L8" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional; el control es por cortinas de seguridad e interlocks de puerta en el perímetro.</t>
+          <t xml:space="preserve">No se requiere EPP adicional; el control real es un dispositivo de control a dos manos en el punto de activación del clampeo.</t>
         </is>
       </c>
       <c r="M8" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOP Operación Kasalis PIXID 500</t>
+          <t xml:space="preserve">16-AT40-3318-00005</t>
         </is>
       </c>
       <c r="N8" s="57" t="inlineStr">
@@ -6692,12 +6692,12 @@
       </c>
       <c r="B9" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operación normal - movimiento del mini-gantry dispensador (3 ejes)</t>
+          <t xml:space="preserve">Operación normal - descarga de material terminado</t>
         </is>
       </c>
       <c r="C9" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El gantry del dispensador se mueve para aplicar el químico (DELO) sobre la pieza en la estación correspondiente</t>
+          <t xml:space="preserve">El operador retira la pieza terminada de la estación de descarga al finalizar el ciclo</t>
         </is>
       </c>
       <c r="D9" s="56" t="inlineStr">
@@ -6722,7 +6722,7 @@
       </c>
       <c r="H9" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="I9" s="57" t="inlineStr">
@@ -6741,12 +6741,12 @@
       </c>
       <c r="L9" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional; el control es por cortinas de seguridad del perímetro.</t>
+          <t xml:space="preserve">No se requiere EPP adicional; el control es por cortinas de seguridad del perímetro (el ciclo automático ya terminó antes de que el operador tenga acceso).</t>
         </is>
       </c>
       <c r="M9" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOP Operación Kasalis PIXID 500</t>
+          <t xml:space="preserve">16-AT40-3318-00005</t>
         </is>
       </c>
       <c r="N9" s="57" t="inlineStr">
@@ -6778,12 +6778,12 @@
       </c>
       <c r="B10" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operación normal - movimiento del mini-gantry PnP (3 ejes, gripper)</t>
+          <t xml:space="preserve">Operación normal - limpieza de la máquina</t>
         </is>
       </c>
       <c r="C10" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El gantry del PnP mueve el gripper para tomar/colocar la pieza entre estaciones</t>
+          <t xml:space="preserve">El operador realiza limpieza rutinaria de la máquina (áreas accesibles con las cortinas/guardas cerradas)</t>
         </is>
       </c>
       <c r="D10" s="56" t="inlineStr">
@@ -6798,7 +6798,7 @@
       </c>
       <c r="F10" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fractura</t>
+          <t xml:space="preserve">Laceración</t>
         </is>
       </c>
       <c r="G10" s="56" t="inlineStr">
@@ -6808,7 +6808,7 @@
       </c>
       <c r="H10" s="57" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">2</t>
         </is>
       </c>
       <c r="I10" s="57" t="inlineStr">
@@ -6827,12 +6827,12 @@
       </c>
       <c r="L10" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional; mismo set de cortinas de seguridad que protege torna-mesa y gantry dispensador.</t>
+          <t xml:space="preserve">No se requiere EPP adicional; el control es por cortinas de seguridad e interlocks de puerta del perímetro.</t>
         </is>
       </c>
       <c r="M10" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOP Operación Kasalis PIXID 500</t>
+          <t xml:space="preserve">16-AT40-3318-00005</t>
         </is>
       </c>
       <c r="N10" s="57" t="inlineStr">
@@ -6864,61 +6864,61 @@
       </c>
       <c r="B11" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Manejo de materiales - carga de pieza en la estación con contacto directo del operador</t>
+          <t xml:space="preserve">Operación normal - manejo de materiales (carga y descarga repetitiva de piezas)</t>
         </is>
       </c>
       <c r="C11" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El operador coloca la pieza en la estación de carga; al hacerlo se activa el pistón de clampeo que asegura la pieza. Es el punto de mayor riesgo de la máquina por el contacto directo del operador con el mecanismo.</t>
+          <t xml:space="preserve">El operador carga y descarga piezas repetidamente en la estación durante el turno</t>
         </is>
       </c>
       <c r="D11" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mecanico</t>
+          <t xml:space="preserve">Ergonomía</t>
         </is>
       </c>
       <c r="E11" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Partes móviles</t>
+          <t xml:space="preserve">Movimientos repetitivos</t>
         </is>
       </c>
       <c r="F11" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Amputación</t>
+          <t xml:space="preserve">Fatiga muscular</t>
         </is>
       </c>
       <c r="G11" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Control</t>
+          <t xml:space="preserve">Influencia</t>
         </is>
       </c>
       <c r="H11" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
-      </c>
-      <c r="I11" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
         </is>
       </c>
+      <c r="I11" s="57" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3</t>
+        </is>
+      </c>
       <c r="J11" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K11" s="107" t="inlineStr">
         <is>
-          <t xml:space="preserve">sensores</t>
+          <t xml:space="preserve">ergonomía</t>
         </is>
       </c>
       <c r="L11" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">No se requiere EPP adicional; el control real es un dispositivo de control a dos manos en el punto de activación del clampeo.</t>
+          <t xml:space="preserve">No se requiere EPP adicional.</t>
         </is>
       </c>
       <c r="M11" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">SOP Operación Kasalis PIXID 500</t>
+          <t xml:space="preserve">16-AT40-3318-00005</t>
         </is>
       </c>
       <c r="N11" s="57" t="inlineStr">
@@ -6928,7 +6928,7 @@
       </c>
       <c r="O11" s="49" t="inlineStr">
         <is>
-          <t xml:space="preserve">3</t>
+          <t xml:space="preserve">4</t>
         </is>
       </c>
       <c r="P11" s="61">
@@ -6950,12 +6950,12 @@
       </c>
       <c r="B12" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Operación normal - dispensación de químico (DELO) y limpieza de boquilla</t>
+          <t xml:space="preserve">Operación normal - dispensación de químico (DELO) cerca de la estación de carga</t>
         </is>
       </c>
       <c r="C12" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El dispensador aplica el químico sobre la pieza; el operador puede tener contacto con residuos durante limpieza de boquilla o cambio de cartucho</t>
+          <t xml:space="preserve">El dispensador aplica el químico sobre la pieza durante el ciclo automático; el operador puede tener contacto ocasional con residuos en la estación de carga/descarga</t>
         </is>
       </c>
       <c r="D12" s="56" t="inlineStr">
@@ -7004,7 +7004,7 @@
       </c>
       <c r="M12" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Evaluación EHS química / SDS del adhesivo DELO</t>
+          <t xml:space="preserve">16-AT40-3318-00005</t>
         </is>
       </c>
       <c r="N12" s="57" t="inlineStr">
@@ -7036,12 +7036,12 @@
       </c>
       <c r="B13" s="55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mantenimiento - intervención con interlocks de puerta desactivados</t>
+          <t xml:space="preserve">Mantenimiento - intervención con interlocks de puerta desactivados (torna-mesa, gantry dispensador, gantry PnP)</t>
         </is>
       </c>
       <c r="C13" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">El personal de mantenimiento coloca el switch de llave en modo Mantenimiento y bloquea el switch general de energía antes de intervenir</t>
+          <t xml:space="preserve">El personal de mantenimiento coloca el switch de llave en modo Mantenimiento y bloquea el switch general de energía antes de intervenir la torna-mesa, el mini-gantry dispensador o el mini-gantry PnP</t>
         </is>
       </c>
       <c r="D13" s="56" t="inlineStr">
@@ -7090,7 +7090,7 @@
       </c>
       <c r="M13" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Procedimiento LOTO de la estación</t>
+          <t xml:space="preserve">16-AT40-3318-00005</t>
         </is>
       </c>
       <c r="N13" s="57" t="inlineStr">
@@ -7176,7 +7176,7 @@
       </c>
       <c r="M14" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Procedimiento LOTO de la estación</t>
+          <t xml:space="preserve">16-AT40-3318-00005</t>
         </is>
       </c>
       <c r="N14" s="57" t="inlineStr">
@@ -7262,7 +7262,7 @@
       </c>
       <c r="M15" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Procedimiento LOTO de la estación</t>
+          <t xml:space="preserve">16-AT40-3318-00005</t>
         </is>
       </c>
       <c r="N15" s="57" t="inlineStr">
@@ -7287,80 +7287,24 @@
       <c r="S15" s="57"/>
     </row>
     <row r="16" spans="1:19" x14ac:dyDescent="0.2">
-      <c r="A16" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rutinario</t>
-        </is>
-      </c>
-      <c r="B16" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Manejo de materiales - carga manual repetitiva de piezas</t>
-        </is>
-      </c>
-      <c r="C16" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">El operador carga piezas repetidamente en la estación durante el turno</t>
-        </is>
-      </c>
-      <c r="D16" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Ergonomía</t>
-        </is>
-      </c>
-      <c r="E16" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Movimientos repetitivos</t>
-        </is>
-      </c>
-      <c r="F16" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Fatiga muscular</t>
-        </is>
-      </c>
-      <c r="G16" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Influencia</t>
-        </is>
-      </c>
-      <c r="H16" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2</t>
-        </is>
-      </c>
-      <c r="I16" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">3</t>
-        </is>
-      </c>
+      <c r="A16" s="55"/>
+      <c r="B16" s="55"/>
+      <c r="C16" s="56"/>
+      <c r="D16" s="56"/>
+      <c r="E16" s="49"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="56"/>
+      <c r="H16" s="57"/>
+      <c r="I16" s="57"/>
       <c r="J16" s="51">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="K16" s="107" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ergonomía</t>
-        </is>
-      </c>
-      <c r="L16" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">No se requiere EPP adicional.</t>
-        </is>
-      </c>
-      <c r="M16" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Evaluación ergonómica de la estación</t>
-        </is>
-      </c>
-      <c r="N16" s="57" t="inlineStr">
-        <is>
-          <t xml:space="preserve">EHS / Automation</t>
-        </is>
-      </c>
-      <c r="O16" s="49" t="inlineStr">
-        <is>
-          <t xml:space="preserve">4</t>
-        </is>
-      </c>
+      <c r="K16" s="107"/>
+      <c r="L16" s="58"/>
+      <c r="M16" s="58"/>
+      <c r="N16" s="57"/>
+      <c r="O16" s="49"/>
       <c r="P16" s="61">
         <f t="shared" si="4"/>
         <v>0</v>

</xml_diff>